<commit_message>
refactor: rebuild petty cash Excel row rendering
</commit_message>
<xml_diff>
--- a/app/assets/工程零用金範本.xlsx
+++ b/app/assets/工程零用金範本.xlsx
@@ -3,22 +3,23 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9204" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="15264" yWindow="0" windowWidth="15552" windowHeight="16656" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="工程零用金" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="__styles__" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'工程零用金'!$C$1:$F$34</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'工程零用金'!$A$1:$F$2</definedName>
   </definedNames>
-  <calcPr calcId="152511" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="新細明體"/>
       <charset val="136"/>
@@ -65,6 +66,11 @@
       <color theme="1"/>
       <sz val="16"/>
     </font>
+    <font>
+      <name val="PMingLiu"/>
+      <color theme="1"/>
+      <sz val="12"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -80,7 +86,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="49">
+  <borders count="52">
     <border>
       <left/>
       <right/>
@@ -566,6 +572,15 @@
       <diagonal/>
     </border>
     <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
       <top style="thick">
@@ -659,15 +674,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -680,6 +686,24 @@
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border/>
+    <border>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -688,7 +712,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -776,118 +800,134 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="49" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -1231,7 +1271,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="22.2"/>
   <cols>
     <col width="20.6640625" customWidth="1" style="1" min="1" max="2"/>
@@ -1242,357 +1282,164 @@
     <col width="8.88671875" customWidth="1" style="1" min="7" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.8" customHeight="1" s="65" thickBot="1">
-      <c r="A1" s="14" t="inlineStr">
+    <row r="1" ht="24" customHeight="1" s="65" thickBot="1">
+      <c r="A1" s="66" t="n"/>
+      <c r="B1" s="67" t="n"/>
+      <c r="C1" s="67" t="n"/>
+      <c r="D1" s="67" t="n"/>
+      <c r="E1" s="67" t="n"/>
+      <c r="F1" s="68" t="n"/>
+    </row>
+    <row r="2" ht="22.8" customHeight="1" s="65">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>類別</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B2" s="15" t="inlineStr">
         <is>
           <t>項目</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C2" s="15" t="inlineStr">
         <is>
           <t>統編</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D2" s="15" t="inlineStr">
         <is>
           <t>發票號碼</t>
         </is>
       </c>
-      <c r="E1" s="15" t="inlineStr">
+      <c r="E2" s="15" t="inlineStr">
         <is>
           <t>細項</t>
         </is>
       </c>
-      <c r="F1" s="16" t="inlineStr">
+      <c r="F2" s="16" t="inlineStr">
         <is>
           <t>金額</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="33" t="n"/>
-      <c r="B2" s="31" t="n"/>
-      <c r="C2" s="48" t="n"/>
-      <c r="D2" s="31" t="n"/>
-      <c r="E2" s="31" t="n"/>
-      <c r="F2" s="30" t="n"/>
-    </row>
-    <row r="3">
-      <c r="C3" s="48" t="n"/>
-      <c r="D3" s="32" t="n"/>
-      <c r="E3" s="31" t="n"/>
-      <c r="F3" s="22" t="n"/>
-    </row>
-    <row r="4">
-      <c r="C4" s="32" t="n"/>
-      <c r="D4" s="32" t="n"/>
-      <c r="E4" s="31" t="n"/>
-      <c r="F4" s="22" t="n"/>
-    </row>
-    <row r="5">
-      <c r="C5" s="48" t="n"/>
-      <c r="D5" s="32" t="n"/>
-      <c r="E5" s="31" t="n"/>
-      <c r="F5" s="22" t="n"/>
-    </row>
-    <row r="6">
-      <c r="C6" s="48" t="n"/>
-      <c r="D6" s="32" t="n"/>
-      <c r="E6" s="31" t="n"/>
-      <c r="F6" s="22" t="n"/>
-    </row>
-    <row r="7">
-      <c r="C7" s="48" t="n"/>
-      <c r="D7" s="32" t="n"/>
-      <c r="E7" s="31" t="n"/>
-      <c r="F7" s="22" t="n"/>
-    </row>
-    <row r="8">
-      <c r="C8" s="48" t="n"/>
-      <c r="D8" s="32" t="n"/>
-      <c r="E8" s="31" t="n"/>
-      <c r="F8" s="22" t="n"/>
-    </row>
-    <row r="9">
-      <c r="C9" s="48" t="n"/>
-      <c r="D9" s="32" t="n"/>
-      <c r="E9" s="31" t="n"/>
-      <c r="F9" s="22" t="n"/>
-    </row>
-    <row r="10">
-      <c r="C10" s="48" t="n"/>
-      <c r="D10" s="32" t="n"/>
-      <c r="E10" s="31" t="n"/>
-      <c r="F10" s="22" t="n"/>
-    </row>
-    <row r="11">
-      <c r="B11" s="32" t="n"/>
-      <c r="C11" s="32" t="n"/>
-      <c r="D11" s="32" t="n"/>
-      <c r="E11" s="32" t="n"/>
-      <c r="F11" s="22" t="n"/>
-    </row>
-    <row r="12">
-      <c r="C12" s="48" t="n"/>
-      <c r="D12" s="36" t="n"/>
-      <c r="E12" s="32" t="n"/>
-      <c r="F12" s="51" t="n"/>
-    </row>
-    <row r="13">
-      <c r="C13" s="48" t="n"/>
-      <c r="D13" s="36" t="n"/>
-      <c r="E13" s="32" t="n"/>
-      <c r="F13" s="51" t="n"/>
-    </row>
-    <row r="14">
-      <c r="C14" s="48" t="n"/>
-      <c r="D14" s="36" t="n"/>
-      <c r="E14" s="32" t="n"/>
-      <c r="F14" s="51" t="n"/>
-    </row>
-    <row r="15">
-      <c r="C15" s="48" t="n"/>
-      <c r="D15" s="36" t="n"/>
-      <c r="E15" s="32" t="n"/>
-      <c r="F15" s="51" t="n"/>
-    </row>
-    <row r="16">
-      <c r="C16" s="31" t="n"/>
-      <c r="D16" s="36" t="n"/>
-      <c r="E16" s="32" t="n"/>
-      <c r="F16" s="51" t="n"/>
-    </row>
-    <row r="17">
-      <c r="C17" s="48" t="n"/>
-      <c r="D17" s="36" t="n"/>
-      <c r="E17" s="32" t="n"/>
-      <c r="F17" s="51" t="n"/>
-    </row>
-    <row r="18">
-      <c r="C18" s="48" t="n"/>
-      <c r="D18" s="36" t="n"/>
-      <c r="E18" s="32" t="n"/>
-      <c r="F18" s="51" t="n"/>
-    </row>
-    <row r="19">
-      <c r="C19" s="48" t="n"/>
-      <c r="D19" s="36" t="n"/>
-      <c r="E19" s="32" t="n"/>
-      <c r="F19" s="51" t="n"/>
-    </row>
-    <row r="20">
-      <c r="C20" s="48" t="n"/>
-      <c r="D20" s="36" t="n"/>
-      <c r="E20" s="32" t="n"/>
-      <c r="F20" s="51" t="n"/>
-    </row>
-    <row r="21">
-      <c r="C21" s="48" t="n"/>
-      <c r="D21" s="36" t="n"/>
-      <c r="E21" s="32" t="n"/>
-      <c r="F21" s="51" t="n"/>
-    </row>
-    <row r="22">
-      <c r="C22" s="48" t="n"/>
-      <c r="D22" s="36" t="n"/>
-      <c r="E22" s="32" t="n"/>
-      <c r="F22" s="51" t="n"/>
-    </row>
-    <row r="23">
-      <c r="C23" s="48" t="n"/>
-      <c r="D23" s="36" t="n"/>
-      <c r="E23" s="32" t="n"/>
-      <c r="F23" s="51" t="n"/>
-    </row>
-    <row r="24" ht="22.8" customHeight="1" s="65" thickBot="1">
-      <c r="C24" s="48" t="n"/>
-      <c r="D24" s="36" t="n"/>
-      <c r="E24" s="32" t="n"/>
-      <c r="F24" s="51" t="n"/>
-    </row>
-    <row r="25" ht="27" customHeight="1" s="65" thickBot="1">
-      <c r="A25" s="37" t="n"/>
-      <c r="F25" s="53" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="56" t="n"/>
-      <c r="B26" s="59" t="n"/>
-      <c r="C26" s="60" t="n"/>
-      <c r="D26" s="60" t="n"/>
-      <c r="E26" s="60" t="n"/>
-      <c r="F26" s="66" t="n"/>
-    </row>
-    <row r="27">
-      <c r="E27" s="32" t="n"/>
-    </row>
-    <row r="28">
-      <c r="C28" s="47" t="n"/>
-      <c r="D28" s="32" t="n"/>
-      <c r="E28" s="32" t="n"/>
-      <c r="F28" s="22" t="n"/>
-    </row>
-    <row r="29">
-      <c r="C29" s="25" t="n"/>
-      <c r="D29" s="32" t="n"/>
-      <c r="E29" s="32" t="n"/>
-      <c r="F29" s="22" t="n"/>
-    </row>
-    <row r="30">
-      <c r="C30" s="48" t="n"/>
-      <c r="D30" s="32" t="n"/>
-      <c r="E30" s="32" t="n"/>
-      <c r="F30" s="22" t="n"/>
-    </row>
-    <row r="31">
-      <c r="C31" s="47" t="n"/>
-      <c r="D31" s="32" t="n"/>
-      <c r="E31" s="32" t="n"/>
-      <c r="F31" s="22" t="n"/>
-    </row>
-    <row r="32">
-      <c r="E32" s="32" t="n"/>
-    </row>
-    <row r="33">
-      <c r="E33" s="32" t="n"/>
-    </row>
-    <row r="34">
-      <c r="E34" s="32" t="n"/>
-    </row>
-    <row r="35">
-      <c r="E35" s="32" t="n"/>
-    </row>
-    <row r="36">
-      <c r="E36" s="32" t="n"/>
-    </row>
-    <row r="37">
-      <c r="C37" s="18" t="n"/>
-      <c r="D37" s="32" t="n"/>
-      <c r="E37" s="32" t="n"/>
-      <c r="F37" s="22" t="n"/>
-    </row>
-    <row r="38">
-      <c r="C38" s="32" t="n"/>
-      <c r="D38" s="32" t="n"/>
-      <c r="E38" s="36" t="n"/>
-      <c r="F38" s="22" t="n"/>
-    </row>
-    <row r="39">
-      <c r="E39" s="36" t="n"/>
-    </row>
-    <row r="40" ht="22.8" customHeight="1" s="65" thickBot="1">
-      <c r="C40" s="62" t="n"/>
-      <c r="D40" s="63" t="n"/>
-      <c r="E40" s="63" t="n"/>
-      <c r="F40" s="64" t="n"/>
-    </row>
-    <row r="41" ht="27" customFormat="1" customHeight="1" s="2" thickBot="1">
-      <c r="A41" s="37" t="n"/>
-      <c r="F41" s="55" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="14" t="n"/>
-      <c r="B42" s="15" t="n"/>
-      <c r="C42" s="31" t="n"/>
-      <c r="D42" s="31" t="n"/>
-      <c r="E42" s="31" t="n"/>
-      <c r="F42" s="30" t="n"/>
-    </row>
-    <row r="43">
-      <c r="C43" s="32" t="n"/>
-      <c r="D43" s="32" t="n"/>
-      <c r="E43" s="32" t="n"/>
-      <c r="F43" s="22" t="n"/>
-    </row>
-    <row r="44">
-      <c r="C44" s="36" t="n"/>
-      <c r="D44" s="36" t="n"/>
-      <c r="E44" s="31" t="n"/>
-      <c r="F44" s="51" t="n"/>
-    </row>
-    <row r="45">
-      <c r="C45" s="36" t="n"/>
-      <c r="D45" s="36" t="n"/>
-      <c r="E45" s="32" t="n"/>
-      <c r="F45" s="51" t="n"/>
-    </row>
-    <row r="46">
-      <c r="C46" s="36" t="n"/>
-      <c r="D46" s="36" t="n"/>
-      <c r="E46" s="32" t="n"/>
-      <c r="F46" s="51" t="n"/>
-    </row>
-    <row r="47">
-      <c r="C47" s="36" t="n"/>
-      <c r="D47" s="36" t="n"/>
-      <c r="E47" s="32" t="n"/>
-      <c r="F47" s="51" t="n"/>
-    </row>
-    <row r="48">
-      <c r="C48" s="36" t="n"/>
-      <c r="D48" s="36" t="n"/>
-      <c r="E48" s="32" t="n"/>
-      <c r="F48" s="51" t="n"/>
-    </row>
-    <row r="49">
-      <c r="C49" s="36" t="n"/>
-      <c r="D49" s="36" t="n"/>
-      <c r="E49" s="36" t="n"/>
-      <c r="F49" s="51" t="n"/>
-    </row>
-    <row r="50">
-      <c r="C50" s="36" t="n"/>
-      <c r="D50" s="36" t="n"/>
-      <c r="E50" s="36" t="n"/>
-      <c r="F50" s="51" t="n"/>
-    </row>
-    <row r="51">
-      <c r="C51" s="36" t="n"/>
-      <c r="D51" s="36" t="n"/>
-      <c r="E51" s="32" t="n"/>
-      <c r="F51" s="51" t="n"/>
-    </row>
-    <row r="52">
-      <c r="C52" s="36" t="n"/>
-      <c r="D52" s="36" t="n"/>
-      <c r="E52" s="32" t="n"/>
-      <c r="F52" s="51" t="n"/>
-    </row>
-    <row r="53" ht="22.8" customHeight="1" s="65" thickBot="1">
-      <c r="C53" s="36" t="n"/>
-      <c r="D53" s="36" t="n"/>
-      <c r="E53" s="36" t="n"/>
-      <c r="F53" s="51" t="n"/>
-    </row>
-    <row r="54" ht="27" customHeight="1" s="65" thickBot="1">
-      <c r="A54" s="37" t="n"/>
-      <c r="F54" s="9" t="n"/>
-    </row>
-    <row r="55" ht="22.8" customHeight="1" s="65" thickBot="1">
-      <c r="A55" s="10" t="n"/>
-      <c r="B55" s="11" t="n"/>
-      <c r="C55" s="11" t="n"/>
-      <c r="D55" s="11" t="n"/>
-      <c r="E55" s="11" t="n"/>
-      <c r="F55" s="12" t="n"/>
-    </row>
-    <row r="56" ht="22.2" customHeight="1" s="65" thickBot="1" thickTop="1">
-      <c r="A56" s="41" t="n"/>
-      <c r="F56" s="41" t="n"/>
-    </row>
-    <row r="57" ht="22.2" customHeight="1" s="65" thickBot="1" thickTop="1"/>
-    <row r="58" ht="22.2" customHeight="1" s="65" thickBot="1" thickTop="1"/>
-    <row r="59" ht="22.8" customHeight="1" s="65" thickTop="1"/>
-    <row r="61" ht="47.4" customHeight="1" s="65"/>
-    <row r="63" ht="19.8" customHeight="1" s="65"/>
-    <row r="65" ht="91.2" customHeight="1" s="65"/>
   </sheetData>
-  <autoFilter ref="C1:F34"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" scale="82" fitToHeight="0" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col hidden="1" width="13" customWidth="1" style="65" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1" s="65">
+      <c r="A1" s="69" t="n"/>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>engineering_title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22.8" customHeight="1" s="65">
+      <c r="A2" s="14" t="n"/>
+      <c r="B2" s="15" t="n"/>
+      <c r="C2" s="15" t="n"/>
+      <c r="D2" s="15" t="n"/>
+      <c r="E2" s="15" t="n"/>
+      <c r="F2" s="16" t="n"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>engineering_header</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" s="65">
+      <c r="A3" s="70" t="n"/>
+      <c r="B3" s="36" t="n"/>
+      <c r="C3" s="36" t="n"/>
+      <c r="D3" s="36" t="n"/>
+      <c r="E3" s="36" t="n"/>
+      <c r="F3" s="22" t="n"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>engineering_data</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="27" customHeight="1" s="65">
+      <c r="A4" s="37" t="n"/>
+      <c r="B4" s="71" t="n"/>
+      <c r="C4" s="71" t="n"/>
+      <c r="D4" s="71" t="n"/>
+      <c r="E4" s="71" t="n"/>
+      <c r="F4" s="30" t="n"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>engineering_subtotal</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22.8" customHeight="1" s="65">
+      <c r="A5" s="10" t="n"/>
+      <c r="B5" s="11" t="n"/>
+      <c r="C5" s="11" t="n"/>
+      <c r="D5" s="11" t="n"/>
+      <c r="E5" s="11" t="n"/>
+      <c r="F5" s="12" t="n"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>engineering_spacer</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22.2" customHeight="1" s="65">
+      <c r="A6" s="40" t="n"/>
+      <c r="B6" s="72" t="n"/>
+      <c r="C6" s="72" t="n"/>
+      <c r="D6" s="72" t="n"/>
+      <c r="E6" s="73" t="n"/>
+      <c r="F6" s="40" t="n"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>engineering_total_top</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22.2" customHeight="1" s="65">
+      <c r="A7" s="74" t="n"/>
+      <c r="E7" s="75" t="n"/>
+      <c r="F7" s="76" t="n"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>engineering_total_middle</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22.2" customHeight="1" s="65">
+      <c r="A8" s="77" t="n"/>
+      <c r="B8" s="78" t="n"/>
+      <c r="C8" s="78" t="n"/>
+      <c r="D8" s="78" t="n"/>
+      <c r="E8" s="79" t="n"/>
+      <c r="F8" s="80" t="n"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>engineering_total_bottom</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: standardize Excel exports and auto-fit columns
</commit_message>
<xml_diff>
--- a/app/assets/工程零用金範本.xlsx
+++ b/app/assets/工程零用金範本.xlsx
@@ -1,141 +1,83 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\workspace\hvac-inventory-work\app\assets\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1282556-51B7-46C4-B919-25B6EA5CDB6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1470" yWindow="1470" windowWidth="23040" windowHeight="11333" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1470" yWindow="1470" windowWidth="23040" windowHeight="11333" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="工程零用金" sheetId="1" r:id="rId1"/>
-    <sheet name="__styles__" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工程零用金" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="__styles__" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">工程零用金!$A$1:$F$2</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'工程零用金'!$A$1:$F$2</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
-  <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
-  <si>
-    <t>類別</t>
-  </si>
-  <si>
-    <t>項目</t>
-  </si>
-  <si>
-    <t>統編</t>
-  </si>
-  <si>
-    <t>發票號碼</t>
-  </si>
-  <si>
-    <t>細項</t>
-  </si>
-  <si>
-    <t>金額</t>
-  </si>
-  <si>
-    <t>engineering_title</t>
-  </si>
-  <si>
-    <t>engineering_header</t>
-  </si>
-  <si>
-    <t>engineering_data</t>
-  </si>
-  <si>
-    <t>engineering_subtotal</t>
-  </si>
-  <si>
-    <t>engineering_spacer</t>
-  </si>
-  <si>
-    <t>engineering_total_top</t>
-  </si>
-  <si>
-    <t>engineering_total_middle</t>
-  </si>
-  <si>
-    <t>engineering_total_bottom</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="7">
     <font>
+      <name val="新細明體"/>
+      <charset val="136"/>
+      <family val="2"/>
+      <color theme="1"/>
       <sz val="12"/>
-      <color theme="1"/>
-      <name val="新細明體"/>
-      <family val="2"/>
-      <charset val="136"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="新細明體"/>
+      <charset val="136"/>
+      <family val="2"/>
       <sz val="9"/>
-      <name val="新細明體"/>
-      <family val="2"/>
-      <charset val="136"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="新細明體"/>
+      <charset val="136"/>
+      <family val="1"/>
+      <b val="1"/>
+      <color theme="1"/>
       <sz val="16"/>
-      <color theme="1"/>
-      <name val="新細明體"/>
-      <family val="1"/>
-      <charset val="136"/>
     </font>
     <font>
-      <b/>
+      <name val="Noto Serif HK Black"/>
+      <charset val="136"/>
+      <family val="1"/>
+      <b val="1"/>
+      <color theme="4" tint="-0.249977111117893"/>
       <sz val="16"/>
-      <color theme="4" tint="-0.249977111117893"/>
-      <name val="Noto Serif HK Black"/>
-      <family val="1"/>
-      <charset val="136"/>
     </font>
     <font>
+      <name val="Noto Serif HK Black"/>
+      <charset val="136"/>
+      <family val="1"/>
+      <color theme="1"/>
       <sz val="30"/>
-      <color theme="1"/>
-      <name val="Noto Serif HK Black"/>
-      <family val="1"/>
-      <charset val="136"/>
     </font>
     <font>
+      <name val="PMingLiu"/>
+      <charset val="136"/>
+      <family val="1"/>
+      <color theme="1"/>
       <sz val="12"/>
-      <color theme="1"/>
-      <name val="PMingLiu"/>
-      <family val="1"/>
-      <charset val="136"/>
     </font>
     <font>
-      <b/>
+      <name val="新細明體"/>
+      <charset val="136"/>
+      <family val="1"/>
+      <b val="1"/>
+      <color theme="1"/>
       <sz val="16"/>
-      <color theme="1"/>
-      <name val="新細明體"/>
-      <family val="1"/>
-      <charset val="136"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -147,7 +89,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="25">
+  <borders count="26">
     <border>
       <left/>
       <right/>
@@ -433,93 +375,163 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="30">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+  <cellXfs count="32">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -785,150 +797,181 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="22.9"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.86328125" defaultRowHeight="22.9"/>
   <cols>
-    <col min="1" max="2" width="20.6640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="15.6640625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="34.6640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="60.46484375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="49.19921875" style="29" customWidth="1"/>
-    <col min="7" max="7" width="8.86328125" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.86328125" style="1"/>
+    <col width="20.6640625" customWidth="1" style="1" min="1" max="2"/>
+    <col width="15.6640625" customWidth="1" style="1" min="3" max="3"/>
+    <col width="34.6640625" customWidth="1" style="1" min="4" max="4"/>
+    <col width="60.46484375" customWidth="1" style="1" min="5" max="5"/>
+    <col width="49.19921875" customWidth="1" style="29" min="6" max="6"/>
+    <col width="8.86328125" customWidth="1" style="1" min="7" max="7"/>
+    <col width="8.86328125" customWidth="1" style="1" min="8" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="24" customHeight="1" thickBot="1">
-      <c r="A1" s="26"/>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="27"/>
+    <row r="1" ht="24" customHeight="1" s="13" thickBot="1">
+      <c r="A1" s="27" t="n"/>
+      <c r="B1" s="30" t="n"/>
+      <c r="C1" s="30" t="n"/>
+      <c r="D1" s="30" t="n"/>
+      <c r="E1" s="30" t="n"/>
+      <c r="F1" s="31" t="n"/>
     </row>
-    <row r="2" spans="1:6" ht="22.8" customHeight="1" thickBot="1">
-      <c r="A2" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="F2" s="28" t="s">
-        <v>5</v>
+    <row r="2" ht="22.8" customHeight="1" s="13" thickBot="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>類別</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>項目</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>統編</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>發票／收據號碼</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>細項</t>
+        </is>
+      </c>
+      <c r="F2" s="28" t="inlineStr">
+        <is>
+          <t>金額</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="82" fitToHeight="0" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="82" fitToHeight="0" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G8"/>
-  <sheetFormatPr defaultRowHeight="16.149999999999999"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16.15"/>
   <cols>
-    <col min="7" max="7" width="13" style="13" hidden="1" customWidth="1"/>
+    <col hidden="1" width="13" customWidth="1" style="13" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="24" customHeight="1">
-      <c r="A1" s="14"/>
-      <c r="G1" t="s">
-        <v>6</v>
+    <row r="1" ht="24" customHeight="1" s="13">
+      <c r="A1" s="14" t="n"/>
+      <c r="G1" s="0" t="inlineStr">
+        <is>
+          <t>engineering_title</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="22.8" customHeight="1">
-      <c r="A2" s="5"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="7"/>
-      <c r="G2" t="s">
-        <v>7</v>
+    <row r="2" ht="22.8" customHeight="1" s="13">
+      <c r="A2" s="5" t="n"/>
+      <c r="B2" s="6" t="n"/>
+      <c r="C2" s="6" t="n"/>
+      <c r="D2" s="6" t="n"/>
+      <c r="E2" s="6" t="n"/>
+      <c r="F2" s="7" t="n"/>
+      <c r="G2" s="0" t="inlineStr">
+        <is>
+          <t>engineering_header</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="22.9">
-      <c r="A3" s="15"/>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="8"/>
-      <c r="G3" t="s">
-        <v>8</v>
+    <row r="3" ht="22.9" customHeight="1" s="13">
+      <c r="A3" s="15" t="n"/>
+      <c r="B3" s="10" t="n"/>
+      <c r="C3" s="10" t="n"/>
+      <c r="D3" s="10" t="n"/>
+      <c r="E3" s="10" t="n"/>
+      <c r="F3" s="8" t="n"/>
+      <c r="G3" s="0" t="inlineStr">
+        <is>
+          <t>engineering_data</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="27" customHeight="1">
-      <c r="A4" s="11"/>
-      <c r="B4" s="16"/>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="9"/>
-      <c r="G4" t="s">
-        <v>9</v>
+    <row r="4" ht="27" customHeight="1" s="13">
+      <c r="A4" s="11" t="n"/>
+      <c r="B4" s="16" t="n"/>
+      <c r="C4" s="16" t="n"/>
+      <c r="D4" s="16" t="n"/>
+      <c r="E4" s="16" t="n"/>
+      <c r="F4" s="9" t="n"/>
+      <c r="G4" s="0" t="inlineStr">
+        <is>
+          <t>engineering_subtotal</t>
+        </is>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="22.8" customHeight="1">
-      <c r="A5" s="2"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="4"/>
-      <c r="G5" t="s">
-        <v>10</v>
+    <row r="5" ht="22.8" customHeight="1" s="13">
+      <c r="A5" s="2" t="n"/>
+      <c r="B5" s="3" t="n"/>
+      <c r="C5" s="3" t="n"/>
+      <c r="D5" s="3" t="n"/>
+      <c r="E5" s="3" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="0" t="inlineStr">
+        <is>
+          <t>engineering_spacer</t>
+        </is>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="22.25" customHeight="1">
-      <c r="A6" s="12"/>
-      <c r="B6" s="17"/>
-      <c r="C6" s="17"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="12"/>
-      <c r="G6" t="s">
-        <v>11</v>
+    <row r="6" ht="22.25" customHeight="1" s="13">
+      <c r="A6" s="12" t="n"/>
+      <c r="B6" s="17" t="n"/>
+      <c r="C6" s="17" t="n"/>
+      <c r="D6" s="17" t="n"/>
+      <c r="E6" s="18" t="n"/>
+      <c r="F6" s="12" t="n"/>
+      <c r="G6" s="0" t="inlineStr">
+        <is>
+          <t>engineering_total_top</t>
+        </is>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="22.25" customHeight="1">
-      <c r="A7" s="19"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="21"/>
-      <c r="G7" t="s">
-        <v>12</v>
+    <row r="7" ht="22.25" customHeight="1" s="13">
+      <c r="A7" s="19" t="n"/>
+      <c r="E7" s="20" t="n"/>
+      <c r="F7" s="21" t="n"/>
+      <c r="G7" s="0" t="inlineStr">
+        <is>
+          <t>engineering_total_middle</t>
+        </is>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="22.25" customHeight="1">
-      <c r="A8" s="22"/>
-      <c r="B8" s="23"/>
-      <c r="C8" s="23"/>
-      <c r="D8" s="23"/>
-      <c r="E8" s="24"/>
-      <c r="F8" s="25"/>
-      <c r="G8" t="s">
-        <v>13</v>
+    <row r="8" ht="22.25" customHeight="1" s="13">
+      <c r="A8" s="22" t="n"/>
+      <c r="B8" s="23" t="n"/>
+      <c r="C8" s="23" t="n"/>
+      <c r="D8" s="23" t="n"/>
+      <c r="E8" s="24" t="n"/>
+      <c r="F8" s="25" t="n"/>
+      <c r="G8" s="0" t="inlineStr">
+        <is>
+          <t>engineering_total_bottom</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>